<commit_message>
Clean national Card Assets names via logo review; record Angle 1 finding
Resolved garbled OCR names (FNBC, Mainstreet FL, Bank of Walker County GA,
Mountain Valley GA, First Security, etc.) and flagged affinity/rewards
programs that are not banks. Angle 1 conclusion: the 75 are out-of-state
community banks + affinity programs, none new in CA; out-of-state applicant
eligibility is not published and needs a Card Assets call to confirm.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LSjV8LuVU5EY9WZi6z4RDo
</commit_message>
<xml_diff>
--- a/SoCal_Equifax_CardAssets_MASTER.xlsx
+++ b/SoCal_Equifax_CardAssets_MASTER.xlsx
@@ -1121,17 +1121,21 @@
       <c r="C13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>0162</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>MERICAN ASS ANGLERS®</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>American Bass Anglers</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Affinity program (not a bank)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1199,17 +1203,21 @@
       <c r="C19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>0210</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>e&amp;. SWAMINARAYAN CREDIT CARD</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Swaminarayan (affinity)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Affinity card (not a bank)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1671,30 +1679,38 @@
       <c r="C55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>1062</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>y, Lop yore 1] REWARDS</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr"/>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>everywhere REWARDS</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Generic rewards logo (not a bank)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>1072</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>y, Lop yore 1] REWARDS</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr"/>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>everywhere REWARDS</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Generic rewards logo (not a bank)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1704,10 +1720,14 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>FINSC COMMUNITY BANKERS</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr"/>
+          <t>FNBC (Community Bankers)</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>AR/LA community bank</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1717,10 +1737,14 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Bat aiystReey COMMUNITY BANK</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr"/>
+          <t>Mainstreet Community Bank of Florida</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1730,7 +1754,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Pear</t>
+          <t>The Union Bank</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr"/>
@@ -1743,10 +1767,14 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>BANK OF WALKER COUNTY</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr"/>
+          <t>Bank of Walker County</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1769,10 +1797,14 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>OUNTAIN ALLEY \ COMMUNITY BANK n of The Piedmont Bank</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr"/>
+          <t>Mountain Valley Community Bank (div. The Piedmont Bank)</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1795,7 +1827,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>1) first security bank</t>
+          <t>First Security Bank</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr"/>
@@ -1840,17 +1872,21 @@
       <c r="C68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>2000</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>ASSOCIATION</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr"/>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>UCA Alumni Association</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Affinity program (not a bank)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -4684,7 +4720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4892,6 +4928,22 @@
       <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Out-of-state eligibility must be verified per bank, not assumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ANGLE 1 FINDING (2026-07-20)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Cleaned all 75 names: they are small out-of-state community banks (AR/GA/FL/etc.) + a few affinity programs. NONE are new CA banks. Out-of-state APPLICANT eligibility is NOT published on the SelectionBusiness pages (they show only products + consent). Definitive answer requires calling Card Assets 800-982-4511 or reading each application's residency terms at the address step. Single-issuer structure (First Arkansas B&amp;T) makes out-of-state acceptance plausible but must be verified per program — do not assume.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark Ojai/Santa Barbara Card Assets lanes defunct; add zombie-page rule
FDIC shows both charters inactive (acquired by Bank of the Sierra, Oct 2017);
their Card Assets pages are ~9-year-old legacy artifacts. Adds the resulting
validation rule (live page != live program) and applies it to the Hanmi lead.
Re-verified First Foundation 0350 live today with all 5 products.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LSjV8LuVU5EY9WZi6z4RDo
</commit_message>
<xml_diff>
--- a/SoCal_Equifax_CardAssets_MASTER.xlsx
+++ b/SoCal_Equifax_CardAssets_MASTER.xlsx
@@ -772,7 +772,7 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>CONFIRMED. Sunflower merger 4/1/26 — apply before legacy lane migrates</t>
+          <t>CONFIRMED. Sunflower merger 4/1/26 — apply before legacy lane migrates | RE-VERIFIED LIVE 2026-07-20 (all 5 products, Apply buttons).</t>
         </is>
       </c>
     </row>
@@ -820,107 +820,107 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>LEAD. Current cards route to Synchrony; call 855-773-8778 to confirm 0092</t>
+          <t>LEAD. Current cards route to Synchrony; call 855-773-8778 to confirm 0092 | CAUTION: Ojai/SB case proves stale Card Assets pages persist ~9 yrs post-merger — a live page does NOT prove a live program. Call is mandatory before relying on 0092.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Santa Barbara Community Bank</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>2002</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Santa Barbara</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Card Assets Mastercard business</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>https://app.thecardservicescenter.com/SelectionBusiness/index/2002</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Live app page</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Equifax (intel)</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Central Coast; division of Ojai Community Bank</t>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>n/a (defunct)</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>DEFUNCT: acquired by Bank of the Sierra (Sierra Bancorp) Oct 2017; charter inactive per FDIC. Card Assets page is a stale legacy artifact (~2015 logo). Bank of the Sierra = Elan.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Ojai Community Bank</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>2250</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Ventura</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Card Assets Mastercard business</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>https://app.thecardservicescenter.com/SelectionBusiness/index/2250</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Live app page</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Equifax (intel)</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Central Coast</t>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>n/a (defunct)</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>DEFUNCT: acquired by Bank of the Sierra (Sierra Bancorp) Oct 2017; charter inactive per FDIC. Card Assets page is a stale legacy artifact (~2015 logo). Bank of the Sierra = Elan.</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4944,6 +4944,22 @@
       <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Cleaned all 75 names: they are small out-of-state community banks (AR/GA/FL/etc.) + a few affinity programs. NONE are new CA banks. Out-of-state APPLICANT eligibility is NOT published on the SelectionBusiness pages (they show only products + consent). Definitive answer requires calling Card Assets 800-982-4511 or reading each application's residency terms at the address step. Single-issuer structure (First Arkansas B&amp;T) makes out-of-state acceptance plausible but must be verified per program — do not assume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>ZOMBIE-PAGE RULE (2026-07-20)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Ojai CB + Santa Barbara CB were acquired by Bank of the Sierra in Oct 2017, yet their Card Assets application pages still load in 2026. Therefore: an index/#### page being live is NOT sufficient evidence of an active program. Every Card Assets lane must be validated against FDIC ACTIVE status + a bank confirmation before use. First Foundation passes (page live + program was active pre-merger); Hanmi requires the call.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Inquiry Data Association method (Tab 8)
Documents how to find out-of-region EQ lenders into CA via inquiry data:
CreditBoards/myFICO credit-pulls DB filtered to CA+Equifax, subtract local
set, grade by recency/volume. Flags self-reported reliability caveat and
that the user's own hard-inquiry history is the highest-grade source to mine.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LSjV8LuVU5EY9WZi6z4RDo
</commit_message>
<xml_diff>
--- a/SoCal_Equifax_CardAssets_MASTER.xlsx
+++ b/SoCal_Equifax_CardAssets_MASTER.xlsx
@@ -15,6 +15,7 @@
     <sheet name="5. Bureau Datapoints" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="6. Out-of-Region Strategy" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="7. Ledger" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="8. Inquiry Data Association" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,6 +47,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="7">
@@ -93,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -120,6 +125,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5274,4 +5282,186 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>INQUIRY DATA ASSOCIATION — finding out-of-region banks that lend into CA</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Principle</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>A hard inquiry on a California applicant's report = proof that lender approved/pulled into CA, regardless of HQ. Filter inquiry data by CA + Equifax to surface out-of-region EQ lenders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>PRIMARY TOOL</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>CreditBoards Credit Pulls Database (creditboards.com/forums) — filter by Consumer State + Credit Reporting Agency + Date + Approval Status. myFICO has an equivalent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>PROCEDURE</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>1. Pull</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Query State=California, Bureau=Equifax -&gt; institution list w/ approval, limit, date</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2. Subtract local</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Cross-ref vs FDIC LA/OC list (Tab 3); remainder = out-of-region lenders into CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>3. Grade</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Weight by recency + volume of DPs; drop stale singletons (bureau practices drift, e.g. First-Citizens EQ-&gt;EX ~2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>4. Merge</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Add survivors to Tab 5 (Bureau Datapoints) w/ source link + COMMUNITY-DP grade; flag those accepting business apps</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>CAVEATS</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Self-reported</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Crowdsourced; treat as COMMUNITY-DP (lead, not fact). WalletHub disputes reliability. Confirm before relying.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>State-specific</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Bureau choice varies by state (Chase/Citi = TransUnion-only in CA). CA filter is mandatory; never generalize national DPs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>BEST SOURCE = OUR OWN DATA</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>User's hard-inquiry spreadsheet record history = real inquiries on real CA reports (higher grade than crowdsourced). ACTION: mine it -&gt; extract institutions -&gt; subtract local -&gt; rank out-of-region lenders by frequency. Awaiting file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>KNOWN CA+EQ SIGNALS (community, unconfirmed)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Discover + Capital One pull EQ in CA (Cap One pulls all 3). Truist/PNC/Citizens noted as frequent EQ pullers (out-of-region, lend into CA) — but big-issuer/no-go overlap; verify per product. Chase/Citi = TransUnion-only in CA (NOT EQ).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Record external inquiry-data sweep results (DoC/myFICO/CreditBoards)
CA+Equifax for out-of-region regional business cards is thin in public
aggregators (self-reported, business-sparse, key sources 403-walled). National
EQ-leaders (PNC/Truist/HSBC/BBVA/Barclays/Discover/CapOne) mostly flip to
EX/TU under CA routing or are user no-gos; PNC is the lone out-of-region EQ
candidate that survives. Reinforces Card Assets as the only state-independent
EQ guarantee; internal inquiry history is the higher-value next lever.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LSjV8LuVU5EY9WZi6z4RDo
</commit_message>
<xml_diff>
--- a/SoCal_Equifax_CardAssets_MASTER.xlsx
+++ b/SoCal_Equifax_CardAssets_MASTER.xlsx
@@ -4514,7 +4514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4716,6 +4716,138 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>PNC Bank</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Equifax (+TU/EX)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>COMMUNITY + user notes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Out-of-region, lends into CA; self-UW. Best-supported out-of-region EQ candidate. Confirm CA routing</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Truist (ex-SunTrust)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Equifax-leaning</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>COMMUNITY (natl)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Out-of-region; on EQ 'leaderboard' nationally; CA routing UNVERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>HSBC</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Equifax-leaning</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>COMMUNITY (natl)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Out-of-region; EQ leaderboard; CA routing UNVERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>BBVA / Barclays</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Equifax-leaning</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>COMMUNITY (natl)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>EQ leaderboard nationally; verify CA + business availability</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Discover / Capital One</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Equifax (consistent in CA)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>COMMUNITY-DP</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Most EQ-consistent even in CA — BUT both are user 2017 NO-GOs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>CA state routing (context)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Mostly EX/TU</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>AGGREGATOR</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>In CA ~1 of 9 tracked issuers pulls EQ; Chase=TU-only, US Bank=EX-only. EQ is the minority bureau in CA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5290,7 +5422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5461,6 +5593,22 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>EXTERNAL SWEEP RESULT (2026-07-20)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Ran DoC, myFICO, CreditBoards refs, uponarriving, aggregators. Public data is THIN for our exact target (out-of-region REGIONAL BUSINESS cards, CA, Equifax): self-reported, sparse for business, richest sources 403-walled. National EQ-leaders (PNC, Truist, HSBC, BBVA, Barclays, Discover, CapOne) mostly (a) flip to EX/TU under CA state-routing or (b) are user no-gos. Only PNC is both out-of-region + EQ + not-no-go + CA-plausible (in user's own notes). CONCLUSION: crowdsourced external route = low yield; Card Assets (First Arkansas B&amp;T) remains the only STATE-INDEPENDENT EQ guarantee. Highest-value remaining lever = INTERNAL (user's own hard-inquiry history).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Bay Area CU batch 3 to Alameda tab
Meriwest CU = Elan (verified, loc 20450) with easy CA/AZ membership and live
online application. Bay Federal CU = self-issued business Visa to $50K but
hard three-county HQ gate. Star One and Self-Help FCU have no business card.
Community Bank of the Bay is defunct — acquired by Commercial Bank of
California 11/1/2024, card program discontinued (was TIB then Elan, never TCM).

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LSjV8LuVU5EY9WZi6z4RDo
</commit_message>
<xml_diff>
--- a/SoCal_Equifax_CardAssets_MASTER.xlsx
+++ b/SoCal_Equifax_CardAssets_MASTER.xlsx
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1940,6 +1940,264 @@
       <c r="I29" s="5" t="inlineStr">
         <is>
           <t>Merged into Nuvision 6/2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Meriwest CU</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>San Jose</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>YES (3 cards)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>ELAN (VERIFIED own-page, loc 20450)</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>TransUnion (Elan rail)</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>YES - onboarding.elancreditcard.com</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>FOM incl. Alameda. EASY outsider path: Financial Fitness Assn, any CA/AZ resident. NOTE: Elan = user NO-GO</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Bay Federal CU</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Capitola</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>YES - Business Visa to $50K</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>SELF-ISSUED (VERIFIED)</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>NO - Formstack lead form/phone</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>HARD GATE: business must be HQ'd Santa Cruz/San Benito/Monterey. No association path. Non-Elan self-issued = worth a bureau call</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Star One CU</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Sunnyvale</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Does not offer business accounts to corps/partnerships at all; sole-prop only (name must contain surname)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Self-Help FCU</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>CU</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Oakland (Alameda)</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>Consumer Mastercard only. EASY $5 membership (Center for Community Self-Help) but no business card</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Community Bank of the Bay</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Oakland (Alameda)</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>DEFUNCT / discontinued</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Historically TIB -&gt; ELAN (never TCM)</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>ACQUIRED by Commercial Bank of California 11/1/2024; bankcbb.com 301-&gt; cbcal.com. Card program discontinued, never resurfaced</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Commercial Bank of California (successor)</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Irvine HQ + Oakland/San Jose/San Mateo/Danville/SF</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr"/>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>Absorbed Community Bank of the Bay. No credit card on successor site (sitemap verified). SoCal bank w/ NorCal footprint</t>
         </is>
       </c>
     </row>
@@ -6575,7 +6833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6988,6 +7246,57 @@
       <c r="C24" s="2" t="inlineStr">
         <is>
           <t>KEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Bay Area CU sweep batch 3 (Star One, Meriwest, Bay Federal, Self-Help, CBB)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>FINDING</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Community Bank of the Bay acquired by Commercial Bank of CA 11/2024; card program dead</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>purge from lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>FINDING</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Meriwest CU = Elan w/ easy CA/AZ membership + live online app (but Elan=no-go)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>noted</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct inquiry-data conclusion; add CreditPulls harvest results
The CreditBoards CreditPulls database is alive and queryable — it moved to
creditboards.com/forums/index.php?/creditpulls/ (old /pulls/ 404s). My earlier
'low yield / inaccessible' conclusion was wrong about accessibility and is
corrected. Harvested results show California is an Experian state for credit
unions: Patelco 72 EX/3 EQ with all 17 CA records Experian, Logix 100% EX,
SchoolsFirst 5/5 CA EX. Equifax-primary CUs exist (DCU 92 EQ, holds for CA
residents) but DCU's business card is restricted to six New England states, so
no Equifax-primary CU offers a business card obtainable from California.
Redwood CU downgraded: zero CreditPulls records, single unverified snippet.
Flags thecreditpeople.com CU list as fabricated.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LSjV8LuVU5EY9WZi6z4RDo
</commit_message>
<xml_diff>
--- a/SoCal_Equifax_CardAssets_MASTER.xlsx
+++ b/SoCal_Equifax_CardAssets_MASTER.xlsx
@@ -6057,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6565,6 +6565,116 @@
       <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Business card NOT LAUNCHED yet ('coming soon')</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Patelco CU (UPGRADED)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>CREDITPULLS n=75</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>72 EX / 3 EQ; ALL 17 CA records Experian. Confirms earlier community-DP</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Logix FCU</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>CREDITPULLS n=49</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>100% Experian</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>SchoolsFirst</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>CREDITPULLS n=5</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>5/5 CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>DCU (Digital FCU)</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>EQUIFAX</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>CREDITPULLS n=100</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>92 EQ. CA residents 15 EQ. BUT business card NOT available in CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Redwood CU (DOWNGRADED)</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Equifax - unverified</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>SINGLE SNIPPET</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Zero CreditPulls records. One myFICO snippet, undated, unloadable</t>
         </is>
       </c>
     </row>
@@ -6833,7 +6943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7297,6 +7407,57 @@
       <c r="C27" s="2" t="inlineStr">
         <is>
           <t>noted</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>CORRECTION</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>CreditPulls DB is ALIVE at creditboards.com/forums/index.php?/creditpulls/ — earlier 'low yield' call was wrong about accessibility</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>FINDING</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>California = EXPERIAN state for credit unions (Patelco/Logix/SchoolsFirst all EX)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>KEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>FINDING</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>No Equifax-primary CU offers a business card obtainable from CA (DCU is EQ but MA/NH/RI/ME/VT/CT only)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>KEY</t>
         </is>
       </c>
     </row>
@@ -7311,7 +7472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7498,6 +7659,257 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>*** CORRECTION + METHOD UNLOCK (2026-07-31) ***</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Earlier I reported the crowdsourced inquiry route as low-yield/inaccessible. That was WRONG about accessibility. The CreditBoards CreditPulls DB is ALIVE and queryable — it MOVED. Dead: creditboards.com/pulls/ (404). LIVE: https://creditboards.com/forums/index.php?/creditpulls/ — ~200k self-reported records, filterable by Consumer State + CRA (EQ/TU/EX) + Approved. Individual record pages show state/bureau/score/limit/date unambiguously.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>QUERY CAVEAT</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>The site's state+CRA bulk filter does NOT partition correctly across pagination (EQ/EX/TU result sets overlapped by ~1,200 of 1,400 records). Bulk filter counts are unreliable — read individual record pages instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>RECALL GAP</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>The CreditPulls search index misses records that demonstrably exist (e.g. 'First Tech' returns 0 despite a live record page). '0 records' = absence of evidence, NOT evidence of absence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>*** HEADLINE FINDING: CALIFORNIA IS AN EXPERIAN STATE FOR CREDIT UNIONS ***</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Patelco</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>72 Experian / 3 Equifax (n=75). ALL 17 California records = Experian, zero exceptions (~2009-2018). STRONG.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Logix FCU</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>49 records, 100% Experian — every state, every CA record</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>SchoolsFirst</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>5/5 California records = Experian</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Nuvision</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>1 CA record = Experian (Jan 2017, thin/stale)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2">
+        <f>&gt; IMPLICATION</f>
+        <v/>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Equifax is genuinely RARE among CA credit unions. This is why Card Assets matters: it is a national single-issuer platform that pulls EQ regardless of state routing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>EQUIFAX-PRIMARY CUs FOUND (none usable from CA)</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>DCU / Digital FCU</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>92 EQ / 5 EX / 3 TU (n=100); CA residents 15 EQ / 2 EX / 1 TU — EQ holds for Californians. BUT business Visa is 'Available in MA, NH, RI, ME, VT and CT' -&gt; UNUSABLE for a CA business</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Alliant CU</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>70 EQ / 23 TU / 5 EX overall, but CA = 8 EQ / 7 TU (mixed, TU dominates recent). NO business card (consumer cashback pulled 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Langley FCU</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>2/2 EQ but dated 2008 &amp; 2015 — thin and stale. Virginia</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Chartway FCU</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>2 EQ + 1 TU, ALL dated May 2005 — worthless</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>PenFed</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>No business credit card at all</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>No Equifax-primary credit union offers a business card a Bay Area business can actually obtain</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr"/>
+      <c r="B40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>REDWOOD CU — downgraded</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>ZERO CreditPulls records exist. The Equifax FICO 5 claim rests on ONE unverified myFICO snippet (thread 6675557), date unknown, page not loadable. TRAP: RCU's site mentions TransUnion VantageScore — that is their SavvyMoney monitoring widget, NOT the application hard pull. Do not read it either way. -&gt; Verify by phone before relying on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr"/>
+      <c r="B42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>FABRICATED SOURCE — DO NOT USE</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>thecreditpeople.com/bureaus/which-credit-unions-pull-only-equifax is AI-generated fabrication: its 'list' names 'XYZ Credit Union', 'ABC Federal Credit Union', 'Lakeview CU', 'Mountain Valley CU', 'Sunrise Federal CU' — institutions that do not exist. It ranks HIGH for exactly these queries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>'21 CUs That Hard Pull Just Equifax'</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Video-only monetized content (MSN/YouTube). Names surfaced: Langley, SECU MD, Virginia CU, Dept of Commerce FCU, Chartway, AOD, DCU, Interior FCU — ALL East Coast/Southeast, NONE California</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Doctor of Credit</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Covers only the 9 big issuers; its 'Smaller Card Issuers' section literally reads 'None'. No credit union data at all</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add distance-ranked Alameda tab with geocoded branch distances
Tab 10 ranks 25 institutions by real distance from City of Alameda, computed
from FDIC geocoded branch coordinates (haversine). Includes rail/underwriter,
bureau with grade, deposits, nearest branch address, branch count, product
names, application links and apply-online status. Colour-coded by rail:
Card Assets/Equifax gold, Elan blue, TCM/TIB purple, other Equifax green.
Nearest Card Assets lane is Sunflower/First Foundation at 3.2 mi (Oakland).

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LSjV8LuVU5EY9WZi6z4RDo
</commit_message>
<xml_diff>
--- a/SoCal_Equifax_CardAssets_MASTER.xlsx
+++ b/SoCal_Equifax_CardAssets_MASTER.xlsx
@@ -17,6 +17,7 @@
     <sheet name="7. Ledger" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="8. Inquiry Data Association" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="9. Alameda - Bay Area" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10. Alameda by DISTANCE" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +54,12 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +96,11 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4DFEC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -104,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -137,6 +147,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2206,6 +2223,1189 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="58" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>DISTANCE-RANKED — measured from City of Alameda CA (37.7652,-122.2416). Nearest branch per institution via FDIC geocoded locations. GOLD=Card Assets/Equifax, BLUE=Elan(TU), PURPLE=TCM/TIB, GREEN=other Equifax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Miles from Alameda CA</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Institution</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Rail / Underwriter</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Bureau</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Deposits ($K)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Nearest branch / location</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>CA branches</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Apply link</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Apply online?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Bank of Marin</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>ELAN</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>TransUnion (rail)</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>2208 S Shore Ctr, Alameda</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Elan business cards</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>bankofmarin.com</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Yes (Elan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Metropolitan Bank</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>TCM Bank, N.A.</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Experian (rail)</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>196224</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>250 E 18th St, Oakland</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>TCM business card</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>https://www.mycommunitycc.com/FROlvrV1uR72/business</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Gateway Bank, F.S.B.</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>TIB, N.A.</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>202316</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>388 9th St, Oakland</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Business No Fee Card; Business Choice Rewards ($49/card)</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>https://www.cardaccount.net/application/e4e363902e/business/new</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>SUNFLOWER BANK (dba First Foundation)</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>*** CARD ASSETS ***</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>EQUIFAX</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr"/>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>323 20th St, OAKLAND</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Platinum Classic/Payback/Preferred, World Elite, World Elite Plus</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>https://app.thecardservicescenter.com/SelectionBusiness/index/0350</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>YES - VERIFIED LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Mechanics Bank</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>ELAN</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>TransUnion (rail)</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>18251541</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>1999 Harrison St, Oakland</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>132</v>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Elan business cards</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>https://www.mymechanics.com/business/loans-credit/business-credit-cards/</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Yes (Elan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Self-Help FCU</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>- (no business card)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Oakland</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>None - consumer Mastercard only</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>self-helpfcu.org</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>United Business Bank</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>NOT DISCLOSED</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>2267047</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>100 Hegenberger Rd, Oakland</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Generic 'Business Credit Card'</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>unitedbusinessbank.com</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>No - request info</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Beneficial State Bank</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>NOT DISCLOSED</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1655342</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>2100 Franklin St, Oakland</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Program exists; no product names published</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>beneficialstatebank.com</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>No - officer contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Summit Bank</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>TIB, N.A.</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>211474</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>2969 Broadway, Oakland</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Standard Card; Preferred Points</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>https://www.summitbanking.com/wp-content/uploads/2019/08/Business-Credit-Card-Application.pdf</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>No - print/branch/fax</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Fremont Bank</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>CorServ/Apex -&gt; Pinnacle Bank TN</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Experian (user notes)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>5269655</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>1480 E 14th St, San Leandro</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Business Platinum / Platinum Rewards / Platinum Low Rate / World Elite MC</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>https://fremontbank.myapexcard.com</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Nuvision CU (ex-Co-op FCU branch)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Self-issued</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Berkeley</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Business Visa</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>nuvisionfederal.com/business-banking/credit-cards</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>No - download/fax/branch</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Avidbank</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>CorServ/Apex (Account Issuer)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>2202730</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>135 Main St, San Francisco</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Credit Cards</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>https://avidbank.myapexcard.com/</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>No - RM only</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Bank of San Francisco</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>ELAN</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>TransUnion (rail)</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>670003</v>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>345 California St, San Francisco</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>myaccountaccess.com (login only)</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco FCU</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>- (no business card)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>sanfranciscofcu.com</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>HANMI BANK</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>*** CARD ASSETS (verify) ***</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>EQUIFAX if live</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>6801918</v>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>7912 Dublin Blvd, DUBLIN</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>Card Assets Mastercard business</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t>https://app.thecardservicescenter.com/SelectionBusiness/index/0092</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>Live page - CALL 855-773-8778</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Provident CU</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Self-issued (VERIFIED)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Redwood City</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Business Rewards Visa; Business Share Secured Visa</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>https://providentcu.org/business/business-credit-cards/apply</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Members only</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Patelco CU</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Self-issued (CFPB-verified)</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>EXPERIAN (72 EX/3 EQ; all 17 CA = EX)</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr"/>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Dublin / Pleasanton (Alameda Cty)</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr"/>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>Business Rewards Mastercard to $40K, no AF</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>https://www.patelco.org/business-banking/business-rewards-card</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>No - Virtual Branch/branch</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>1st United CU</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>- (no business card)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Pleasanton (Alameda Cty)</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>None - consumer only</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>1stunitedcu.org</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Star One CU</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>- (no business card)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Sunnyvale</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>No business accounts for corps/partnerships</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>starone.org</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Meriwest CU</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>ELAN (VERIFIED, loc 20450)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>TransUnion (rail)</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>San Jose</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Business Cash Preferred; Smart Business Rewards; Business Real Rewards</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>https://onboarding.elancreditcard.com/gateway/v1/applications/partner-prefill?locationCode=20450&amp;offerId=R3MV2VDWD2&amp;preparerType=customer</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>YES - easy CA/AZ membership</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Tech CU</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>- (no business card)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>San Jose</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>None - business debit only</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>techcu.com</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="n">
+        <v>37</v>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Pinnacle Bank (Gilroy)</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>TIB, N.A.</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>823506</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>1999 S Bascom Ave, Campbell</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>Mastercard business; Preferred Points</t>
+        </is>
+      </c>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>pinnaclebankca.com</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Redwood CU</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Self-issued (CFPB-verified)</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>EQUIFAX FICO 5 (UNVERIFIED - 0 CreditPulls records)</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr"/>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>Santa Rosa</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr"/>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>Business Visa Platinum / Preferred / Select</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>https://www.redwoodcu.org/business/cards/business-visa-platinum/</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>Yes - BUT Alameda OUTSIDE field of membership</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Bay Federal CU</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Self-issued (VERIFIED)</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>UNKNOWN - could be EQ</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr"/>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Capitola</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr"/>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>Business Visa to $50K, no AF</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>https://www.bayfed.com/business/visa-credit</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>No - lead form. HARD GATE: Santa Cruz/San Benito/Monterey HQ only</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Golden 1</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Unknown - not published</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Experian (consumer)</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Sacramento (statewide)</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Business Cash Rewards - COMING SOON, not launched</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.golden1.com/business-services/business-credit-cards</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>No - not launched</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>